<commit_message>
Update product import file to remove category information
Modify metadata to reflect the updated product import file lacking category data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: c2f211a7-1115-4266-9d02-0dd5e7945c87
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b9664fb9-ca19-4ca7-87ae-4304eecc4dc8
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2efb9ae1-c32a-4281-a068-894d3f42b551/c2f211a7-1115-4266-9d02-0dd5e7945c87/3RBKiqw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/products_import.xlsx
+++ b/products_import.xlsx
@@ -509,11 +509,7 @@
           <t>Eyelashes - Cluster Lasher</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Eyelashes</t>
-        </is>
-      </c>
+      <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="3" t="n">
         <v>100</v>
       </c>
@@ -528,11 +524,7 @@
           <t>Eyelashes - Striper Lashes</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Eyelashes</t>
-        </is>
-      </c>
+      <c r="B3" s="4" t="inlineStr"/>
       <c r="C3" s="5" t="n">
         <v>50</v>
       </c>
@@ -547,11 +539,7 @@
           <t>Eyelashes - Striper Small Lashes</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Eyelashes</t>
-        </is>
-      </c>
+      <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="3" t="n">
         <v>30</v>
       </c>
@@ -566,11 +554,7 @@
           <t>Foundation - Green Tea</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Foundations</t>
-        </is>
-      </c>
+      <c r="B5" s="4" t="inlineStr"/>
       <c r="C5" s="5" t="n">
         <v>70</v>
       </c>
@@ -585,11 +569,7 @@
           <t>Foundation - Sleek</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Foundations</t>
-        </is>
-      </c>
+      <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="3" t="n">
         <v>50</v>
       </c>
@@ -604,11 +584,7 @@
           <t>Foundation - Blackopal</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Foundations</t>
-        </is>
-      </c>
+      <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="5" t="n">
         <v>60</v>
       </c>
@@ -623,11 +599,7 @@
           <t>Primers</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Face</t>
-        </is>
-      </c>
+      <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="3" t="n">
         <v>60</v>
       </c>
@@ -642,11 +614,7 @@
           <t>Concealors</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Face</t>
-        </is>
-      </c>
+      <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="5" t="n">
         <v>70</v>
       </c>
@@ -661,11 +629,7 @@
           <t>Liquid Matte Lipsticks</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="3" t="n">
         <v>20</v>
       </c>
@@ -680,11 +644,7 @@
           <t>Irene Lipstick</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="5" t="n">
         <v>60</v>
       </c>
@@ -699,11 +659,7 @@
           <t>Normal Matte Lipstick</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="3" t="n">
         <v>200</v>
       </c>
@@ -718,11 +674,7 @@
           <t>Vaseline Lipbalm</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="5" t="n">
         <v>35</v>
       </c>
@@ -737,11 +689,7 @@
           <t>Roll-on Lipbalm</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="3" t="n">
         <v>30</v>
       </c>
@@ -756,11 +704,7 @@
           <t>Romantic Lipbalm</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="5" t="n">
         <v>30</v>
       </c>
@@ -775,11 +719,7 @@
           <t>Strawberry Lipbalm</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="3" t="n">
         <v>30</v>
       </c>
@@ -794,11 +734,7 @@
           <t>Simple Lipbalm</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="5" t="n">
         <v>20</v>
       </c>
@@ -813,11 +749,7 @@
           <t>Lipglosser - Magic Lipgloss</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="3" t="n">
         <v>30</v>
       </c>
@@ -832,11 +764,7 @@
           <t>Lipglosser - Adoge Cithas Lipgloss</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B19" s="4" t="inlineStr"/>
       <c r="C19" s="5" t="n">
         <v>80</v>
       </c>
@@ -851,11 +779,7 @@
           <t>Lipglosser - Absolute Lipgloss</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="n">
         <v>30</v>
       </c>
@@ -870,11 +794,7 @@
           <t>Lipglosser - Squeeze n Shine</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B21" s="4" t="inlineStr"/>
       <c r="C21" s="5" t="n">
         <v>30</v>
       </c>
@@ -889,11 +809,7 @@
           <t>Lipglosser - Mood Lipgloss</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="3" t="n">
         <v>30</v>
       </c>
@@ -908,11 +824,7 @@
           <t>Lipglosser - VC Small Lipgloss</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B23" s="4" t="inlineStr"/>
       <c r="C23" s="5" t="n">
         <v>15</v>
       </c>
@@ -927,11 +839,7 @@
           <t>Lip Oil - Normal</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="3" t="n">
         <v>70</v>
       </c>
@@ -946,11 +854,7 @@
           <t>Lip Oil - With a Charm</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Lip Care</t>
-        </is>
-      </c>
+      <c r="B25" s="4" t="inlineStr"/>
       <c r="C25" s="5" t="n">
         <v>200</v>
       </c>
@@ -965,11 +869,7 @@
           <t>Men Wallets</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="3" t="n">
         <v>200</v>
       </c>
@@ -984,11 +884,7 @@
           <t>Ladies Wallets</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B27" s="4" t="inlineStr"/>
       <c r="C27" s="5" t="n">
         <v>100</v>
       </c>
@@ -1003,11 +899,7 @@
           <t>Anklets</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="3" t="n">
         <v>50</v>
       </c>
@@ -1022,11 +914,7 @@
           <t>Tinkles</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B29" s="4" t="inlineStr"/>
       <c r="C29" s="5" t="n">
         <v>50</v>
       </c>
@@ -1041,11 +929,7 @@
           <t>Key Holders</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="3" t="n">
         <v>200</v>
       </c>
@@ -1060,11 +944,7 @@
           <t>Phone Charms</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B31" s="4" t="inlineStr"/>
       <c r="C31" s="5" t="n">
         <v>150</v>
       </c>
@@ -1079,11 +959,7 @@
           <t>Nosering - Metallic</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="3" t="n">
         <v>10</v>
       </c>
@@ -1098,11 +974,7 @@
           <t>Nosering - Plastic</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B33" s="4" t="inlineStr"/>
       <c r="C33" s="5" t="n">
         <v>10</v>
       </c>
@@ -1117,11 +989,7 @@
           <t>Plastic Earrings</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="3" t="n">
         <v>10</v>
       </c>
@@ -1136,11 +1004,7 @@
           <t>Body Piercing Stainless</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B35" s="4" t="inlineStr"/>
       <c r="C35" s="5" t="n">
         <v>30</v>
       </c>
@@ -1155,11 +1019,7 @@
           <t>Pocket Mirror</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="3" t="n">
         <v>20</v>
       </c>
@@ -1174,11 +1034,7 @@
           <t>Pocket Mirror (Small)</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B37" s="4" t="inlineStr"/>
       <c r="C37" s="5" t="n">
         <v>50</v>
       </c>
@@ -1193,11 +1049,7 @@
           <t>Pocket Mirror (Big)</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="3" t="n">
         <v>5</v>
       </c>
@@ -1212,11 +1064,7 @@
           <t>Gift Boxes / Watches</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B39" s="4" t="inlineStr"/>
       <c r="C39" s="5" t="n">
         <v>100</v>
       </c>
@@ -1231,11 +1079,7 @@
           <t>Gift Boxes</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="3" t="n">
         <v>150</v>
       </c>
@@ -1250,11 +1094,7 @@
           <t>Gift Bags (Small)</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B41" s="4" t="inlineStr"/>
       <c r="C41" s="5" t="n">
         <v>30</v>
       </c>
@@ -1269,11 +1109,7 @@
           <t>Gift Bags (Medium)</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="3" t="n">
         <v>100</v>
       </c>
@@ -1288,11 +1124,7 @@
           <t>Gift Bags (Big)</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B43" s="4" t="inlineStr"/>
       <c r="C43" s="5" t="n">
         <v>150</v>
       </c>
@@ -1307,11 +1139,7 @@
           <t>Sunglasses - Kids</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="3" t="n">
         <v>30</v>
       </c>
@@ -1326,11 +1154,7 @@
           <t>Sunglasses - Frames</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B45" s="4" t="inlineStr"/>
       <c r="C45" s="5" t="n">
         <v>110</v>
       </c>
@@ -1345,11 +1169,7 @@
           <t>Sunglasses - Mens</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B46" s="2" t="inlineStr"/>
       <c r="C46" s="3" t="n">
         <v>110</v>
       </c>
@@ -1364,11 +1184,7 @@
           <t>Sunglasses - Ladies</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B47" s="4" t="inlineStr"/>
       <c r="C47" s="5" t="n">
         <v>100</v>
       </c>
@@ -1383,11 +1199,7 @@
           <t>Sunglasses - Old Skool</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Accessories</t>
-        </is>
-      </c>
+      <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="3" t="n">
         <v>120</v>
       </c>
@@ -1402,11 +1214,7 @@
           <t>Hairbonnet with Strings</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B49" s="4" t="inlineStr"/>
       <c r="C49" s="5" t="n">
         <v>70</v>
       </c>
@@ -1421,11 +1229,7 @@
           <t>Hair Bonnet without Strings</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B50" s="2" t="inlineStr"/>
       <c r="C50" s="3" t="n">
         <v>50</v>
       </c>
@@ -1440,11 +1244,7 @@
           <t>Wig Caps</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B51" s="4" t="inlineStr"/>
       <c r="C51" s="5" t="n">
         <v>20</v>
       </c>
@@ -1459,11 +1259,7 @@
           <t>Headbands - Material Big</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B52" s="2" t="inlineStr"/>
       <c r="C52" s="3" t="n">
         <v>70</v>
       </c>
@@ -1478,11 +1274,7 @@
           <t>Headbands - Material Small</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B53" s="4" t="inlineStr"/>
       <c r="C53" s="5" t="n">
         <v>35</v>
       </c>
@@ -1497,11 +1289,7 @@
           <t>Pushback - Metallic</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B54" s="2" t="inlineStr"/>
       <c r="C54" s="3" t="n">
         <v>70</v>
       </c>
@@ -1516,11 +1304,7 @@
           <t>Pushback - Crystals</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B55" s="4" t="inlineStr"/>
       <c r="C55" s="5" t="n">
         <v>100</v>
       </c>
@@ -1535,11 +1319,7 @@
           <t>Pushback - Pins</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B56" s="2" t="inlineStr"/>
       <c r="C56" s="3" t="n">
         <v>60</v>
       </c>
@@ -1554,11 +1334,7 @@
           <t>Kids Pushbacks</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B57" s="4" t="inlineStr"/>
       <c r="C57" s="5" t="n">
         <v>25</v>
       </c>
@@ -1573,11 +1349,7 @@
           <t>Fascinators</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B58" s="2" t="inlineStr"/>
       <c r="C58" s="3" t="n">
         <v>350</v>
       </c>
@@ -1592,11 +1364,7 @@
           <t>Hair Ribbons</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B59" s="4" t="inlineStr"/>
       <c r="C59" s="5" t="n">
         <v>100</v>
       </c>
@@ -1611,11 +1379,7 @@
           <t>Material (Branche)</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" s="3" t="n">
         <v>100</v>
       </c>
@@ -1630,11 +1394,7 @@
           <t>Haircharms</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B61" s="4" t="inlineStr"/>
       <c r="C61" s="5" t="n">
         <v>10</v>
       </c>
@@ -1649,11 +1409,7 @@
           <t>Moana Clips (Small)</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B62" s="2" t="inlineStr"/>
       <c r="C62" s="3" t="n">
         <v>15</v>
       </c>
@@ -1668,11 +1424,7 @@
           <t>Oval Clips</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B63" s="4" t="inlineStr"/>
       <c r="C63" s="5" t="n">
         <v>15</v>
       </c>
@@ -1687,11 +1439,7 @@
           <t>Fancy Metallic Clips</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B64" s="2" t="inlineStr"/>
       <c r="C64" s="3" t="n">
         <v>15</v>
       </c>
@@ -1706,11 +1454,7 @@
           <t>Mouth Clips</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B65" s="4" t="inlineStr"/>
       <c r="C65" s="5" t="n">
         <v>30</v>
       </c>
@@ -1725,11 +1469,7 @@
           <t>Arrow Clip</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B66" s="2" t="inlineStr"/>
       <c r="C66" s="3" t="n">
         <v>30</v>
       </c>
@@ -1744,11 +1484,7 @@
           <t>Donut Band</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B67" s="4" t="inlineStr"/>
       <c r="C67" s="5" t="n">
         <v>50</v>
       </c>
@@ -1763,11 +1499,7 @@
           <t>Bronches (Small)</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B68" s="2" t="inlineStr"/>
       <c r="C68" s="3" t="n">
         <v>100</v>
       </c>
@@ -1782,11 +1514,7 @@
           <t>Bronches (Medium)</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B69" s="4" t="inlineStr"/>
       <c r="C69" s="5" t="n">
         <v>30</v>
       </c>
@@ -1801,11 +1529,7 @@
           <t>Hairband (Small)</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B70" s="2" t="inlineStr"/>
       <c r="C70" s="3" t="n">
         <v>50</v>
       </c>
@@ -1820,11 +1544,7 @@
           <t>Hairband - Medium (Korea)</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B71" s="4" t="inlineStr"/>
       <c r="C71" s="5" t="n">
         <v>15</v>
       </c>
@@ -1839,11 +1559,7 @@
           <t>Hairband (Big)</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B72" s="2" t="inlineStr"/>
       <c r="C72" s="3" t="n">
         <v>15</v>
       </c>
@@ -1858,11 +1574,7 @@
           <t>Bobby Pin / Hair Pins</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B73" s="4" t="inlineStr"/>
       <c r="C73" s="5" t="n">
         <v>5</v>
       </c>
@@ -1877,11 +1589,7 @@
           <t>Bobby Pin (Big)</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>Hair Accessories</t>
-        </is>
-      </c>
+      <c r="B74" s="2" t="inlineStr"/>
       <c r="C74" s="3" t="n">
         <v>30</v>
       </c>
@@ -1896,11 +1604,7 @@
           <t>Hair Brush (Small)</t>
         </is>
       </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B75" s="4" t="inlineStr"/>
       <c r="C75" s="5" t="n">
         <v>150</v>
       </c>
@@ -1915,11 +1619,7 @@
           <t>Hair Brush (Big)</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="3" t="n">
         <v>200</v>
       </c>
@@ -1934,11 +1634,7 @@
           <t>Grey Hair Dye Pen</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B77" s="4" t="inlineStr"/>
       <c r="C77" s="5" t="n">
         <v>160</v>
       </c>
@@ -1953,11 +1649,7 @@
           <t>Hairgel - Movit</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B78" s="2" t="inlineStr"/>
       <c r="C78" s="3" t="n">
         <v>350</v>
       </c>
@@ -1972,11 +1664,7 @@
           <t>Hairgel - Sofree Free Gel</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B79" s="4" t="inlineStr"/>
       <c r="C79" s="5" t="n">
         <v>170</v>
       </c>
@@ -1991,11 +1679,7 @@
           <t>Hairgel - Nice n Lovely</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="3" t="n">
         <v>160</v>
       </c>
@@ -2010,11 +1694,7 @@
           <t>Dexe Hair Shampoo</t>
         </is>
       </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B81" s="4" t="inlineStr"/>
       <c r="C81" s="5" t="n">
         <v>30</v>
       </c>
@@ -2029,11 +1709,7 @@
           <t>Bonding Glue (Small)</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="3" t="n">
         <v>100</v>
       </c>
@@ -2048,11 +1724,7 @@
           <t>Bonding Glue (Big)</t>
         </is>
       </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B83" s="4" t="inlineStr"/>
       <c r="C83" s="5" t="n">
         <v>120</v>
       </c>
@@ -2067,11 +1739,7 @@
           <t>Hair Cutters (Small)</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="3" t="n">
         <v>20</v>
       </c>
@@ -2086,11 +1754,7 @@
           <t>Hair Cutters (Big)</t>
         </is>
       </c>
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B85" s="4" t="inlineStr"/>
       <c r="C85" s="5" t="n">
         <v>30</v>
       </c>
@@ -2105,11 +1769,7 @@
           <t>Hair Comb - Tail Comb</t>
         </is>
       </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B86" s="2" t="inlineStr"/>
       <c r="C86" s="3" t="n">
         <v>10</v>
       </c>
@@ -2124,11 +1784,7 @@
           <t>Hair Comb - 3 in 1</t>
         </is>
       </c>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B87" s="4" t="inlineStr"/>
       <c r="C87" s="5" t="n">
         <v>20</v>
       </c>
@@ -2143,11 +1799,7 @@
           <t>Hair Comb - Alex Comb</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B88" s="2" t="inlineStr"/>
       <c r="C88" s="3" t="n">
         <v>25</v>
       </c>
@@ -2162,11 +1814,7 @@
           <t>Hair Comb - 2 in 1</t>
         </is>
       </c>
-      <c r="B89" s="4" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B89" s="4" t="inlineStr"/>
       <c r="C89" s="5" t="n">
         <v>30</v>
       </c>
@@ -2181,11 +1829,7 @@
           <t>Subane</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Hair Care</t>
-        </is>
-      </c>
+      <c r="B90" s="2" t="inlineStr"/>
       <c r="C90" s="3" t="n">
         <v>50</v>
       </c>
@@ -2200,11 +1844,7 @@
           <t>Bathing Gloves</t>
         </is>
       </c>
-      <c r="B91" s="4" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B91" s="4" t="inlineStr"/>
       <c r="C91" s="5" t="n">
         <v>80</v>
       </c>
@@ -2219,11 +1859,7 @@
           <t>Body Scrubber Rope</t>
         </is>
       </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B92" s="2" t="inlineStr"/>
       <c r="C92" s="3" t="n">
         <v>50</v>
       </c>
@@ -2238,11 +1874,7 @@
           <t>Foot Scrubbers</t>
         </is>
       </c>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B93" s="4" t="inlineStr"/>
       <c r="C93" s="5" t="n">
         <v>80</v>
       </c>
@@ -2257,11 +1889,7 @@
           <t>Asante Soap</t>
         </is>
       </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B94" s="2" t="inlineStr"/>
       <c r="C94" s="3" t="n">
         <v>60</v>
       </c>
@@ -2276,11 +1904,7 @@
           <t>Pumice Stones</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B95" s="4" t="inlineStr"/>
       <c r="C95" s="5" t="n">
         <v>100</v>
       </c>
@@ -2295,11 +1919,7 @@
           <t>Signature Body Splash (Small 59ml)</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B96" s="2" t="inlineStr"/>
       <c r="C96" s="3" t="n">
         <v>100</v>
       </c>
@@ -2314,11 +1934,7 @@
           <t>Signature Body Splash (Big 236ml)</t>
         </is>
       </c>
-      <c r="B97" s="4" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B97" s="4" t="inlineStr"/>
       <c r="C97" s="5" t="n">
         <v>200</v>
       </c>
@@ -2333,11 +1949,7 @@
           <t>Dear Ladys</t>
         </is>
       </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="3" t="n">
         <v>300</v>
       </c>
@@ -2352,11 +1964,7 @@
           <t>Body Mists</t>
         </is>
       </c>
-      <c r="B99" s="4" t="inlineStr">
-        <is>
-          <t>Body Care</t>
-        </is>
-      </c>
+      <c r="B99" s="4" t="inlineStr"/>
       <c r="C99" s="5" t="n">
         <v>300</v>
       </c>
@@ -2371,11 +1979,7 @@
           <t>Tumeric Oils</t>
         </is>
       </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B100" s="2" t="inlineStr"/>
       <c r="C100" s="3" t="n">
         <v>200</v>
       </c>
@@ -2390,11 +1994,7 @@
           <t>Egyptian Serum</t>
         </is>
       </c>
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B101" s="4" t="inlineStr"/>
       <c r="C101" s="5" t="n">
         <v>250</v>
       </c>
@@ -2409,11 +2009,7 @@
           <t>Moroccan Serum</t>
         </is>
       </c>
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B102" s="2" t="inlineStr"/>
       <c r="C102" s="3" t="n">
         <v>250</v>
       </c>
@@ -2428,11 +2024,7 @@
           <t>Dr Rashel Serum</t>
         </is>
       </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B103" s="4" t="inlineStr"/>
       <c r="C103" s="5" t="n">
         <v>250</v>
       </c>
@@ -2447,11 +2039,7 @@
           <t>Estelin Sunscreen</t>
         </is>
       </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="3" t="n">
         <v>250</v>
       </c>
@@ -2466,11 +2054,7 @@
           <t>Dr Rashel Sunscreen</t>
         </is>
       </c>
-      <c r="B105" s="4" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B105" s="4" t="inlineStr"/>
       <c r="C105" s="5" t="n">
         <v>250</v>
       </c>
@@ -2485,11 +2069,7 @@
           <t>Vitamin C Serum</t>
         </is>
       </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="3" t="n">
         <v>300</v>
       </c>
@@ -2504,11 +2084,7 @@
           <t>Rose Water</t>
         </is>
       </c>
-      <c r="B107" s="4" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B107" s="4" t="inlineStr"/>
       <c r="C107" s="5" t="n">
         <v>150</v>
       </c>
@@ -2523,11 +2099,7 @@
           <t>Aloe Vera Gel (Small)</t>
         </is>
       </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B108" s="2" t="inlineStr"/>
       <c r="C108" s="3" t="n">
         <v>120</v>
       </c>
@@ -2542,11 +2114,7 @@
           <t>Aloe Vera Gel (Medium)</t>
         </is>
       </c>
-      <c r="B109" s="4" t="inlineStr">
-        <is>
-          <t>Skin Care</t>
-        </is>
-      </c>
+      <c r="B109" s="4" t="inlineStr"/>
       <c r="C109" s="5" t="n">
         <v>200</v>
       </c>
@@ -2561,11 +2129,7 @@
           <t>Kajal Eyeliner</t>
         </is>
       </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B110" s="2" t="inlineStr"/>
       <c r="C110" s="3" t="n">
         <v>40</v>
       </c>
@@ -2580,11 +2144,7 @@
           <t>Make Up Set (Small)</t>
         </is>
       </c>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B111" s="4" t="inlineStr"/>
       <c r="C111" s="5" t="n">
         <v>100</v>
       </c>
@@ -2599,11 +2159,7 @@
           <t>Make Up Set (Big)</t>
         </is>
       </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B112" s="2" t="inlineStr"/>
       <c r="C112" s="3" t="n">
         <v>150</v>
       </c>
@@ -2618,11 +2174,7 @@
           <t>Concealor Brush One Sided</t>
         </is>
       </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B113" s="4" t="inlineStr"/>
       <c r="C113" s="5" t="n">
         <v>20</v>
       </c>
@@ -2637,11 +2189,7 @@
           <t>Concealor Brush Two Sided</t>
         </is>
       </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B114" s="2" t="inlineStr"/>
       <c r="C114" s="3" t="n">
         <v>50</v>
       </c>
@@ -2656,11 +2204,7 @@
           <t>Duthan Mascara</t>
         </is>
       </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B115" s="4" t="inlineStr"/>
       <c r="C115" s="5" t="n">
         <v>30</v>
       </c>
@@ -2675,11 +2219,7 @@
           <t>2 in 1 Mascara</t>
         </is>
       </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B116" s="2" t="inlineStr"/>
       <c r="C116" s="3" t="n">
         <v>25</v>
       </c>
@@ -2694,11 +2234,7 @@
           <t>Make Up Sponge (Round)</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B117" s="4" t="inlineStr"/>
       <c r="C117" s="5" t="n">
         <v>20</v>
       </c>
@@ -2713,11 +2249,7 @@
           <t>Make Up Sponge 2 in 1</t>
         </is>
       </c>
-      <c r="B118" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B118" s="2" t="inlineStr"/>
       <c r="C118" s="3" t="n">
         <v>15</v>
       </c>
@@ -2732,11 +2264,7 @@
           <t>Lady Blue</t>
         </is>
       </c>
-      <c r="B119" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B119" s="4" t="inlineStr"/>
       <c r="C119" s="5" t="n">
         <v>50</v>
       </c>
@@ -2751,11 +2279,7 @@
           <t>Lock Sponge</t>
         </is>
       </c>
-      <c r="B120" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B120" s="2" t="inlineStr"/>
       <c r="C120" s="3" t="n">
         <v>120</v>
       </c>
@@ -2770,11 +2294,7 @@
           <t>Eyeshadow (5 in 1)</t>
         </is>
       </c>
-      <c r="B121" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B121" s="4" t="inlineStr"/>
       <c r="C121" s="5" t="n">
         <v>250</v>
       </c>
@@ -2789,11 +2309,7 @@
           <t>Eyeshadow Pallet</t>
         </is>
       </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B122" s="2" t="inlineStr"/>
       <c r="C122" s="3" t="n">
         <v>400</v>
       </c>
@@ -2808,11 +2324,7 @@
           <t>Beauty Blender</t>
         </is>
       </c>
-      <c r="B123" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B123" s="4" t="inlineStr"/>
       <c r="C123" s="5" t="n">
         <v>40</v>
       </c>
@@ -2827,11 +2339,7 @@
           <t>Twizers</t>
         </is>
       </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B124" s="2" t="inlineStr"/>
       <c r="C124" s="3" t="n">
         <v>50</v>
       </c>
@@ -2846,11 +2354,7 @@
           <t>Concealer Brush Small</t>
         </is>
       </c>
-      <c r="B125" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B125" s="4" t="inlineStr"/>
       <c r="C125" s="5" t="n">
         <v>30</v>
       </c>
@@ -2865,11 +2369,7 @@
           <t>Etaloner Pencil</t>
         </is>
       </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B126" s="2" t="inlineStr"/>
       <c r="C126" s="3" t="n">
         <v>30</v>
       </c>
@@ -2884,11 +2384,7 @@
           <t>Cappenci - Normal</t>
         </is>
       </c>
-      <c r="B127" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B127" s="4" t="inlineStr"/>
       <c r="C127" s="5" t="n">
         <v>20</v>
       </c>
@@ -2903,11 +2399,7 @@
           <t>Cappenci - Bold/Liner</t>
         </is>
       </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B128" s="2" t="inlineStr"/>
       <c r="C128" s="3" t="n">
         <v>35</v>
       </c>
@@ -2922,11 +2414,7 @@
           <t>Compact Powder - Sleek Pod (Single)</t>
         </is>
       </c>
-      <c r="B129" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B129" s="4" t="inlineStr"/>
       <c r="C129" s="5" t="n">
         <v>10</v>
       </c>
@@ -2941,11 +2429,7 @@
           <t>Compact Powder - Milani Pods</t>
         </is>
       </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B130" s="2" t="inlineStr"/>
       <c r="C130" s="3" t="n">
         <v>200</v>
       </c>
@@ -2960,11 +2444,7 @@
           <t>Compact Powder - A Face</t>
         </is>
       </c>
-      <c r="B131" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B131" s="4" t="inlineStr"/>
       <c r="C131" s="5" t="n">
         <v>150</v>
       </c>
@@ -2979,11 +2459,7 @@
           <t>Compact Powder - Green Tea</t>
         </is>
       </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B132" s="2" t="inlineStr"/>
       <c r="C132" s="3" t="n">
         <v>50</v>
       </c>
@@ -2998,11 +2474,7 @@
           <t>Compact Powder - Sleek 2 in 1</t>
         </is>
       </c>
-      <c r="B133" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B133" s="4" t="inlineStr"/>
       <c r="C133" s="5" t="n">
         <v>130</v>
       </c>
@@ -3017,11 +2489,7 @@
           <t>Compact Powder - Roseleaf (Small)</t>
         </is>
       </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B134" s="2" t="inlineStr"/>
       <c r="C134" s="3" t="n">
         <v>130</v>
       </c>
@@ -3036,11 +2504,7 @@
           <t>Compact Powder - Roseleaf (Medium)</t>
         </is>
       </c>
-      <c r="B135" s="4" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B135" s="4" t="inlineStr"/>
       <c r="C135" s="5" t="n">
         <v>50</v>
       </c>
@@ -3055,11 +2519,7 @@
           <t>Compact Powder - Roseleaf (Big)</t>
         </is>
       </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t>Cosmetics</t>
-        </is>
-      </c>
+      <c r="B136" s="2" t="inlineStr"/>
       <c r="C136" s="3" t="n">
         <v>70</v>
       </c>
@@ -3074,11 +2534,7 @@
           <t>Nail Files (Big)</t>
         </is>
       </c>
-      <c r="B137" s="4" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B137" s="4" t="inlineStr"/>
       <c r="C137" s="5" t="n">
         <v>50</v>
       </c>
@@ -3093,11 +2549,7 @@
           <t>Nail Files (Small)</t>
         </is>
       </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B138" s="2" t="inlineStr"/>
       <c r="C138" s="3" t="n">
         <v>30</v>
       </c>
@@ -3112,11 +2564,7 @@
           <t>Nail Brusher</t>
         </is>
       </c>
-      <c r="B139" s="4" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B139" s="4" t="inlineStr"/>
       <c r="C139" s="5" t="n">
         <v>30</v>
       </c>
@@ -3131,11 +2579,7 @@
           <t>Nail Glue - Brush On</t>
         </is>
       </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B140" s="2" t="inlineStr"/>
       <c r="C140" s="3" t="n">
         <v>60</v>
       </c>
@@ -3150,11 +2594,7 @@
           <t>Nail Glue - Yoo</t>
         </is>
       </c>
-      <c r="B141" s="4" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B141" s="4" t="inlineStr"/>
       <c r="C141" s="5" t="n">
         <v>160</v>
       </c>
@@ -3169,11 +2609,7 @@
           <t>Nail Glue - Small</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B142" s="2" t="inlineStr"/>
       <c r="C142" s="3" t="n">
         <v>15</v>
       </c>
@@ -3188,11 +2624,7 @@
           <t>Qutex (Small)</t>
         </is>
       </c>
-      <c r="B143" s="4" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B143" s="4" t="inlineStr"/>
       <c r="C143" s="5" t="n">
         <v>15</v>
       </c>
@@ -3207,11 +2639,7 @@
           <t>Qutex (Big)</t>
         </is>
       </c>
-      <c r="B144" s="2" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B144" s="2" t="inlineStr"/>
       <c r="C144" s="3" t="n">
         <v>30</v>
       </c>
@@ -3226,11 +2654,7 @@
           <t>Sticker Nails</t>
         </is>
       </c>
-      <c r="B145" s="4" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B145" s="4" t="inlineStr"/>
       <c r="C145" s="5" t="n">
         <v>30</v>
       </c>
@@ -3245,11 +2669,7 @@
           <t>Tips</t>
         </is>
       </c>
-      <c r="B146" s="2" t="inlineStr">
-        <is>
-          <t>Nail Care</t>
-        </is>
-      </c>
+      <c r="B146" s="2" t="inlineStr"/>
       <c r="C146" s="3" t="n">
         <v>20</v>
       </c>
@@ -3264,11 +2684,7 @@
           <t>Caflon Earring Original</t>
         </is>
       </c>
-      <c r="B147" s="4" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B147" s="4" t="inlineStr"/>
       <c r="C147" s="5" t="n">
         <v>70</v>
       </c>
@@ -3283,11 +2699,7 @@
           <t>Caflon Earring Fake</t>
         </is>
       </c>
-      <c r="B148" s="2" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B148" s="2" t="inlineStr"/>
       <c r="C148" s="3" t="n">
         <v>20</v>
       </c>
@@ -3302,11 +2714,7 @@
           <t>Magnetic Earrings</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B149" s="4" t="inlineStr"/>
       <c r="C149" s="5" t="n">
         <v>35</v>
       </c>
@@ -3321,11 +2729,7 @@
           <t>Earrings - Loops</t>
         </is>
       </c>
-      <c r="B150" s="2" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B150" s="2" t="inlineStr"/>
       <c r="C150" s="3" t="n">
         <v>15</v>
       </c>
@@ -3340,11 +2744,7 @@
           <t>Earrings - Stud</t>
         </is>
       </c>
-      <c r="B151" s="4" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B151" s="4" t="inlineStr"/>
       <c r="C151" s="5" t="n">
         <v>15</v>
       </c>
@@ -3359,11 +2759,7 @@
           <t>Earrings - Hanging</t>
         </is>
       </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B152" s="2" t="inlineStr"/>
       <c r="C152" s="3" t="n">
         <v>30</v>
       </c>
@@ -3378,11 +2774,7 @@
           <t>Earrings - Chunky</t>
         </is>
       </c>
-      <c r="B153" s="4" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B153" s="4" t="inlineStr"/>
       <c r="C153" s="5" t="n">
         <v>100</v>
       </c>
@@ -3397,11 +2789,7 @@
           <t>Earrings - Coated</t>
         </is>
       </c>
-      <c r="B154" s="2" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B154" s="2" t="inlineStr"/>
       <c r="C154" s="3" t="n">
         <v>100</v>
       </c>
@@ -3416,11 +2804,7 @@
           <t>Earrings - Stainless</t>
         </is>
       </c>
-      <c r="B155" s="4" t="inlineStr">
-        <is>
-          <t>Earrings</t>
-        </is>
-      </c>
+      <c r="B155" s="4" t="inlineStr"/>
       <c r="C155" s="5" t="n">
         <v>30</v>
       </c>
@@ -3435,11 +2819,7 @@
           <t>Chains (Giver)</t>
         </is>
       </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B156" s="2" t="inlineStr"/>
       <c r="C156" s="3" t="n">
         <v>100</v>
       </c>
@@ -3454,11 +2834,7 @@
           <t>Gold Earrings Ladies</t>
         </is>
       </c>
-      <c r="B157" s="4" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B157" s="4" t="inlineStr"/>
       <c r="C157" s="5" t="n">
         <v>100</v>
       </c>
@@ -3473,11 +2849,7 @@
           <t>Bracelet (Charms Stainless)</t>
         </is>
       </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B158" s="2" t="inlineStr"/>
       <c r="C158" s="3" t="n">
         <v>150</v>
       </c>
@@ -3492,11 +2864,7 @@
           <t>Gold Chain Mens</t>
         </is>
       </c>
-      <c r="B159" s="4" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B159" s="4" t="inlineStr"/>
       <c r="C159" s="5" t="n">
         <v>200</v>
       </c>
@@ -3511,11 +2879,7 @@
           <t>Fancy Chain Ladies</t>
         </is>
       </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B160" s="2" t="inlineStr"/>
       <c r="C160" s="3" t="n">
         <v>120</v>
       </c>
@@ -3530,11 +2894,7 @@
           <t>Earring and Chain Set</t>
         </is>
       </c>
-      <c r="B161" s="4" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B161" s="4" t="inlineStr"/>
       <c r="C161" s="5" t="n">
         <v>150</v>
       </c>
@@ -3549,11 +2909,7 @@
           <t>Rings - Mid Rings</t>
         </is>
       </c>
-      <c r="B162" s="2" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B162" s="2" t="inlineStr"/>
       <c r="C162" s="3" t="n">
         <v>30</v>
       </c>
@@ -3568,11 +2924,7 @@
           <t>Rings - Engagement Ring</t>
         </is>
       </c>
-      <c r="B163" s="4" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B163" s="4" t="inlineStr"/>
       <c r="C163" s="5" t="n">
         <v>35</v>
       </c>
@@ -3587,11 +2939,7 @@
           <t>Rings - Wedding Ring</t>
         </is>
       </c>
-      <c r="B164" s="2" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B164" s="2" t="inlineStr"/>
       <c r="C164" s="3" t="n">
         <v>50</v>
       </c>
@@ -3606,11 +2954,7 @@
           <t>Rings - Chunky Rings</t>
         </is>
       </c>
-      <c r="B165" s="4" t="inlineStr">
-        <is>
-          <t>Jewellery</t>
-        </is>
-      </c>
+      <c r="B165" s="4" t="inlineStr"/>
       <c r="C165" s="5" t="n">
         <v>150</v>
       </c>
@@ -3625,11 +2969,7 @@
           <t>Smart Collections Perfumer</t>
         </is>
       </c>
-      <c r="B166" s="2" t="inlineStr">
-        <is>
-          <t>Perfumes</t>
-        </is>
-      </c>
+      <c r="B166" s="2" t="inlineStr"/>
       <c r="C166" s="3" t="n">
         <v>120</v>
       </c>
@@ -3644,11 +2984,7 @@
           <t>Crown Perfumes</t>
         </is>
       </c>
-      <c r="B167" s="4" t="inlineStr">
-        <is>
-          <t>Perfumes</t>
-        </is>
-      </c>
+      <c r="B167" s="4" t="inlineStr"/>
       <c r="C167" s="5" t="n">
         <v>100</v>
       </c>
@@ -3663,11 +2999,7 @@
           <t>Pen Spray (Ceriflone)</t>
         </is>
       </c>
-      <c r="B168" s="2" t="inlineStr">
-        <is>
-          <t>Perfumes</t>
-        </is>
-      </c>
+      <c r="B168" s="2" t="inlineStr"/>
       <c r="C168" s="3" t="n">
         <v>75</v>
       </c>
@@ -3682,11 +3014,7 @@
           <t>Invisible Bra</t>
         </is>
       </c>
-      <c r="B169" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B169" s="4" t="inlineStr"/>
       <c r="C169" s="5" t="n">
         <v>150</v>
       </c>
@@ -3701,11 +3029,7 @@
           <t>Bra Straps</t>
         </is>
       </c>
-      <c r="B170" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B170" s="2" t="inlineStr"/>
       <c r="C170" s="3" t="n">
         <v>30</v>
       </c>
@@ -3720,11 +3044,7 @@
           <t>Handkerchiefs</t>
         </is>
       </c>
-      <c r="B171" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B171" s="4" t="inlineStr"/>
       <c r="C171" s="5" t="n">
         <v>30</v>
       </c>
@@ -3739,11 +3059,7 @@
           <t>Belts - Slim Ladies</t>
         </is>
       </c>
-      <c r="B172" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B172" s="2" t="inlineStr"/>
       <c r="C172" s="3" t="n">
         <v>70</v>
       </c>
@@ -3758,11 +3074,7 @@
           <t>Belts - Bacon Ladies</t>
         </is>
       </c>
-      <c r="B173" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B173" s="4" t="inlineStr"/>
       <c r="C173" s="5" t="n">
         <v>110</v>
       </c>
@@ -3777,11 +3089,7 @@
           <t>Belts - Men Belts</t>
         </is>
       </c>
-      <c r="B174" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B174" s="2" t="inlineStr"/>
       <c r="C174" s="3" t="n">
         <v>120</v>
       </c>
@@ -3796,11 +3104,7 @@
           <t>Belts - Elastic Belts</t>
         </is>
       </c>
-      <c r="B175" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B175" s="4" t="inlineStr"/>
       <c r="C175" s="5" t="n">
         <v>130</v>
       </c>
@@ -3815,11 +3119,7 @@
           <t>Panties - Kids</t>
         </is>
       </c>
-      <c r="B176" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B176" s="2" t="inlineStr"/>
       <c r="C176" s="3" t="n">
         <v>150</v>
       </c>
@@ -3834,11 +3134,7 @@
           <t>Panties - G-Strings</t>
         </is>
       </c>
-      <c r="B177" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B177" s="4" t="inlineStr"/>
       <c r="C177" s="5" t="n">
         <v>160</v>
       </c>
@@ -3853,11 +3149,7 @@
           <t>Panties - Thongs</t>
         </is>
       </c>
-      <c r="B178" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B178" s="2" t="inlineStr"/>
       <c r="C178" s="3" t="n">
         <v>150</v>
       </c>
@@ -3872,11 +3164,7 @@
           <t>Panties - Normals</t>
         </is>
       </c>
-      <c r="B179" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B179" s="4" t="inlineStr"/>
       <c r="C179" s="5" t="n">
         <v>150</v>
       </c>
@@ -3891,11 +3179,7 @@
           <t>Ankle Socks</t>
         </is>
       </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B180" s="2" t="inlineStr"/>
       <c r="C180" s="3" t="n">
         <v>30</v>
       </c>
@@ -3910,11 +3194,7 @@
           <t>Ankle Socks Cottons</t>
         </is>
       </c>
-      <c r="B181" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B181" s="4" t="inlineStr"/>
       <c r="C181" s="5" t="n">
         <v>35</v>
       </c>
@@ -3929,11 +3209,7 @@
           <t>Fishnet Stockings</t>
         </is>
       </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B182" s="2" t="inlineStr"/>
       <c r="C182" s="3" t="n">
         <v>120</v>
       </c>
@@ -3948,11 +3224,7 @@
           <t>Normal Stockings (Mtumike)</t>
         </is>
       </c>
-      <c r="B183" s="4" t="inlineStr">
-        <is>
-          <t>Clothing</t>
-        </is>
-      </c>
+      <c r="B183" s="4" t="inlineStr"/>
       <c r="C183" s="5" t="n">
         <v>50</v>
       </c>
@@ -3967,11 +3239,7 @@
           <t>Watches (Wrist)</t>
         </is>
       </c>
-      <c r="B184" s="2" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
+      <c r="B184" s="2" t="inlineStr"/>
       <c r="C184" s="3" t="n">
         <v>10</v>
       </c>
@@ -3986,11 +3254,7 @@
           <t>Magnetic Watches</t>
         </is>
       </c>
-      <c r="B185" s="4" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
+      <c r="B185" s="4" t="inlineStr"/>
       <c r="C185" s="5" t="n">
         <v>165</v>
       </c>
@@ -4005,11 +3269,7 @@
           <t>Rubber Watches</t>
         </is>
       </c>
-      <c r="B186" s="2" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
+      <c r="B186" s="2" t="inlineStr"/>
       <c r="C186" s="3" t="n">
         <v>130</v>
       </c>
@@ -4024,11 +3284,7 @@
           <t>Metallic Watches</t>
         </is>
       </c>
-      <c r="B187" s="4" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
+      <c r="B187" s="4" t="inlineStr"/>
       <c r="C187" s="5" t="n">
         <v>250</v>
       </c>
@@ -4043,11 +3299,7 @@
           <t>Kids Watches</t>
         </is>
       </c>
-      <c r="B188" s="2" t="inlineStr">
-        <is>
-          <t>Watches</t>
-        </is>
-      </c>
+      <c r="B188" s="2" t="inlineStr"/>
       <c r="C188" s="3" t="n">
         <v>100</v>
       </c>
@@ -4062,11 +3314,7 @@
           <t>Razorblades</t>
         </is>
       </c>
-      <c r="B189" s="4" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
+      <c r="B189" s="4" t="inlineStr"/>
       <c r="C189" s="5" t="n">
         <v>3</v>
       </c>
@@ -4081,11 +3329,7 @@
           <t>Durex</t>
         </is>
       </c>
-      <c r="B190" s="2" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
+      <c r="B190" s="2" t="inlineStr"/>
       <c r="C190" s="3" t="n">
         <v>100</v>
       </c>
@@ -4100,11 +3344,7 @@
           <t>Portable Fan (Small)</t>
         </is>
       </c>
-      <c r="B191" s="4" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
+      <c r="B191" s="4" t="inlineStr"/>
       <c r="C191" s="5" t="n">
         <v>250</v>
       </c>
@@ -4119,11 +3359,7 @@
           <t>Portable Fan (Big)</t>
         </is>
       </c>
-      <c r="B192" s="2" t="inlineStr">
-        <is>
-          <t>Electronics</t>
-        </is>
-      </c>
+      <c r="B192" s="2" t="inlineStr"/>
       <c r="C192" s="3" t="n">
         <v>300</v>
       </c>
@@ -4138,11 +3374,7 @@
           <t>Sling Bag - Fluffy Sling</t>
         </is>
       </c>
-      <c r="B193" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B193" s="4" t="inlineStr"/>
       <c r="C193" s="5" t="n">
         <v>300</v>
       </c>
@@ -4157,11 +3389,7 @@
           <t>Sling Bag with a Ribbon</t>
         </is>
       </c>
-      <c r="B194" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B194" s="2" t="inlineStr"/>
       <c r="C194" s="3" t="n">
         <v>400</v>
       </c>
@@ -4176,11 +3404,7 @@
           <t>Min Min Small Sling Bag</t>
         </is>
       </c>
-      <c r="B195" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B195" s="4" t="inlineStr"/>
       <c r="C195" s="5" t="n">
         <v>550</v>
       </c>
@@ -4195,11 +3419,7 @@
           <t>2 in 1 Sling Bag (Leather)</t>
         </is>
       </c>
-      <c r="B196" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B196" s="2" t="inlineStr"/>
       <c r="C196" s="3" t="n">
         <v>1000</v>
       </c>
@@ -4214,11 +3434,7 @@
           <t>Sling Bag (Plain)</t>
         </is>
       </c>
-      <c r="B197" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B197" s="4" t="inlineStr"/>
       <c r="C197" s="5" t="n">
         <v>700</v>
       </c>
@@ -4233,11 +3449,7 @@
           <t>Unisex Sling Bag</t>
         </is>
       </c>
-      <c r="B198" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B198" s="2" t="inlineStr"/>
       <c r="C198" s="3" t="n">
         <v>250</v>
       </c>
@@ -4252,11 +3464,7 @@
           <t>Waist Bag (Small)</t>
         </is>
       </c>
-      <c r="B199" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B199" s="4" t="inlineStr"/>
       <c r="C199" s="5" t="n">
         <v>100</v>
       </c>
@@ -4271,11 +3479,7 @@
           <t>Waist Bag (Big)</t>
         </is>
       </c>
-      <c r="B200" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B200" s="2" t="inlineStr"/>
       <c r="C200" s="3" t="n">
         <v>300</v>
       </c>
@@ -4290,11 +3494,7 @@
           <t>Student Tote Bags</t>
         </is>
       </c>
-      <c r="B201" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B201" s="4" t="inlineStr"/>
       <c r="C201" s="5" t="n">
         <v>500</v>
       </c>
@@ -4309,11 +3509,7 @@
           <t>Travelling Bags</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B202" s="2" t="inlineStr"/>
       <c r="C202" s="3" t="n">
         <v>500</v>
       </c>
@@ -4328,11 +3524,7 @@
           <t>Dolla Bag</t>
         </is>
       </c>
-      <c r="B203" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B203" s="4" t="inlineStr"/>
       <c r="C203" s="5" t="n">
         <v>500</v>
       </c>
@@ -4347,11 +3539,7 @@
           <t>2 in 1 Bag Tote Bag</t>
         </is>
       </c>
-      <c r="B204" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B204" s="2" t="inlineStr"/>
       <c r="C204" s="3" t="n">
         <v>400</v>
       </c>
@@ -4366,11 +3554,7 @@
           <t>Tote Bag with a Matching Hat</t>
         </is>
       </c>
-      <c r="B205" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B205" s="4" t="inlineStr"/>
       <c r="C205" s="5" t="n">
         <v>400</v>
       </c>
@@ -4385,11 +3569,7 @@
           <t>Queen Bags</t>
         </is>
       </c>
-      <c r="B206" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B206" s="2" t="inlineStr"/>
       <c r="C206" s="3" t="n">
         <v>350</v>
       </c>
@@ -4404,11 +3584,7 @@
           <t>Straw Bag / Same Bag with a Hat</t>
         </is>
       </c>
-      <c r="B207" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B207" s="4" t="inlineStr"/>
       <c r="C207" s="5" t="n">
         <v>1100</v>
       </c>
@@ -4423,11 +3599,7 @@
           <t>Jute Bag / Woven Bag</t>
         </is>
       </c>
-      <c r="B208" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B208" s="2" t="inlineStr"/>
       <c r="C208" s="3" t="n">
         <v>300</v>
       </c>
@@ -4442,11 +3614,7 @@
           <t>Partitioned Tote Bags</t>
         </is>
       </c>
-      <c r="B209" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B209" s="4" t="inlineStr"/>
       <c r="C209" s="5" t="n">
         <v>600</v>
       </c>
@@ -4461,11 +3629,7 @@
           <t>Plain Partitioned Bag (Medium)</t>
         </is>
       </c>
-      <c r="B210" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B210" s="2" t="inlineStr"/>
       <c r="C210" s="3" t="n">
         <v>650</v>
       </c>
@@ -4480,11 +3644,7 @@
           <t>Summer Bags (Vibes)</t>
         </is>
       </c>
-      <c r="B211" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B211" s="4" t="inlineStr"/>
       <c r="C211" s="5" t="n">
         <v>500</v>
       </c>
@@ -4499,11 +3659,7 @@
           <t>Mothers Bag</t>
         </is>
       </c>
-      <c r="B212" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B212" s="2" t="inlineStr"/>
       <c r="C212" s="3" t="n">
         <v>1100</v>
       </c>
@@ -4518,11 +3674,7 @@
           <t>GA Tote Bag</t>
         </is>
       </c>
-      <c r="B213" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B213" s="4" t="inlineStr"/>
       <c r="C213" s="5" t="n">
         <v>1100</v>
       </c>
@@ -4537,11 +3689,7 @@
           <t>Fendi Tote Bag</t>
         </is>
       </c>
-      <c r="B214" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B214" s="2" t="inlineStr"/>
       <c r="C214" s="3" t="n">
         <v>1000</v>
       </c>
@@ -4556,11 +3704,7 @@
           <t>Official Bag 2 in 1</t>
         </is>
       </c>
-      <c r="B215" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B215" s="4" t="inlineStr"/>
       <c r="C215" s="5" t="n">
         <v>1200</v>
       </c>
@@ -4575,11 +3719,7 @@
           <t>Minmin Bag Medium (Original)</t>
         </is>
       </c>
-      <c r="B216" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B216" s="2" t="inlineStr"/>
       <c r="C216" s="3" t="n">
         <v>1200</v>
       </c>
@@ -4594,11 +3734,7 @@
           <t>Coach Leather Bag</t>
         </is>
       </c>
-      <c r="B217" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B217" s="4" t="inlineStr"/>
       <c r="C217" s="5" t="n">
         <v>1100</v>
       </c>
@@ -4613,11 +3749,7 @@
           <t>Burberry Bag</t>
         </is>
       </c>
-      <c r="B218" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B218" s="2" t="inlineStr"/>
       <c r="C218" s="3" t="n">
         <v>750</v>
       </c>
@@ -4632,11 +3764,7 @@
           <t>Chain Tote Bag</t>
         </is>
       </c>
-      <c r="B219" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B219" s="4" t="inlineStr"/>
       <c r="C219" s="5" t="n">
         <v>750</v>
       </c>
@@ -4651,11 +3779,7 @@
           <t>3 in 1 Official Bag</t>
         </is>
       </c>
-      <c r="B220" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B220" s="2" t="inlineStr"/>
       <c r="C220" s="3" t="n">
         <v>1000</v>
       </c>
@@ -4670,11 +3794,7 @@
           <t>5 in 1 Bags</t>
         </is>
       </c>
-      <c r="B221" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B221" s="4" t="inlineStr"/>
       <c r="C221" s="5" t="n">
         <v>1800</v>
       </c>
@@ -4689,11 +3809,7 @@
           <t>4 in 1 Bags</t>
         </is>
       </c>
-      <c r="B222" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B222" s="2" t="inlineStr"/>
       <c r="C222" s="3" t="n">
         <v>1700</v>
       </c>
@@ -4708,11 +3824,7 @@
           <t>Monkey Bag Flowered</t>
         </is>
       </c>
-      <c r="B223" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B223" s="4" t="inlineStr"/>
       <c r="C223" s="5" t="n">
         <v>650</v>
       </c>
@@ -4727,11 +3839,7 @@
           <t>Monkey Bag Plain</t>
         </is>
       </c>
-      <c r="B224" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B224" s="2" t="inlineStr"/>
       <c r="C224" s="3" t="n">
         <v>1000</v>
       </c>
@@ -4746,11 +3854,7 @@
           <t>Minmin Big Bag</t>
         </is>
       </c>
-      <c r="B225" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B225" s="4" t="inlineStr"/>
       <c r="C225" s="5" t="n">
         <v>700</v>
       </c>
@@ -4765,11 +3869,7 @@
           <t>Cellophone Bag</t>
         </is>
       </c>
-      <c r="B226" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B226" s="2" t="inlineStr"/>
       <c r="C226" s="3" t="n">
         <v>300</v>
       </c>
@@ -4784,11 +3884,7 @@
           <t>Cello Phone Bag (Small)</t>
         </is>
       </c>
-      <c r="B227" s="4" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
+      <c r="B227" s="4" t="inlineStr"/>
       <c r="C227" s="5" t="n">
         <v>250</v>
       </c>

</xml_diff>